<commit_message>
31 new thoughts (ids 605-635) with a 763-day calendar loop (days to 2 March 2027 unchanged, all rules pass over 40 years), glossary cards for the 10 new thinkers, their books and concepts; two smoother openings; handover for the build in exports/
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XtUBtsHEVvdoDDiuP88LhW
</commit_message>
<xml_diff>
--- a/content/glossary.xlsx
+++ b/content/glossary.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Read me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Schools" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Core concepts" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Other terms" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Map cards" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Coverage" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Removed" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schools" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core concepts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other terms" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Map cards" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Schools'!$A$1:$I$13</definedName>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -468,7 +468,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The Thinking Place glossary, updated 18 October 2026</t>
+          <t>The Thinking Place glossary, updated 28 October 2026</t>
         </is>
       </c>
     </row>
@@ -507,7 +507,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -540,6 +539,14 @@
       <c r="A12" t="inlineStr">
         <is>
           <t>'Appears as' lists the words that open a card. Avoid commas inside a single term: the list is split on commas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>28 October 2026: entries for the 10 new thinkers (ids 605–635), their books and new concepts, marked New (green); path, concept and map cards that now include them are marked Updated. Checked against Wikipedia on 28 October 2026. The Coverage sheet has not been recounted yet.</t>
         </is>
       </c>
     </row>
@@ -760,12 +767,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Moral thought from the 17th to 19th centuries that put reason, evidence and freedom at the centre: Descartes' method of doubt, Spinoza's freedom through understanding, Hume and Adam Smith on feeling, Kant's duty, Mill's greatest happiness, and the case for women's minds made by Émilie du Châtelet and Mary Wollstonecraft.</t>
+          <t>Moral and political thought from the 17th to 19th centuries that put reason, evidence and freedom at the centre: Hobbes and Locke on why we need government, Descartes' method of doubt, Spinoza's freedom through understanding, Hume and Adam Smith on feeling, Voltaire's tolerance, Rousseau and Diderot on nature and the passions, Kant's duty, Mill's greatest happiness, and the case for women's minds made by Émilie du Châtelet and Mary Wollstonecraft.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Descartes, Spinoza, Hume, Adam Smith, Émilie du Châtelet, Kant, Mary Wollstonecraft, Mill</t>
+          <t>Descartes, Hobbes, Spinoza, Locke, Hume, Voltaire, Émilie du Châtelet, Adam Smith, Rousseau, Diderot, Kant, Mary Wollstonecraft, Mill</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -795,7 +802,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Replaces the Duty Ethics and Utilitarianism cards. Descartes, Adam Smith and du Châtelet added since 15 October.</t>
+          <t>28 Oct 2026: Hobbes, Locke, Voltaire, Rousseau and Diderot added.</t>
         </is>
       </c>
     </row>
@@ -854,12 +861,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Writers who explored how to live in personal prose and poetry rather than in systems: Petrarch and Erasmus, who revived ancient wisdom; Montaigne's essays and La Rochefoucauld's maxims; and the American Transcendentalists and poets of the 1800s, who trusted intuition, nature and self-reliance.</t>
+          <t>Writers who explored how to live in personal prose and poetry rather than in systems: Petrarch and Erasmus, who revived ancient wisdom; Machiavelli's hard look at power; the essays of Montaigne and Bacon; the French moralists La Rochefoucauld, La Bruyère, Vauvenargues and Chamfort; and the American Transcendentalists and poets of the 1800s, who trusted intuition, nature and self-reliance.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Petrarch, Erasmus, Montaigne, La Rochefoucauld, Emerson, Margaret Fuller, Thoreau, Emily Dickinson, George Eliot</t>
+          <t>Petrarch, Erasmus, Machiavelli, Montaigne, Francis Bacon, La Rochefoucauld, La Bruyère, Vauvenargues, Chamfort, Emerson, Margaret Fuller, Thoreau, Emily Dickinson, George Eliot</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -889,7 +896,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>New name (was 'Essayists and Transcendentalists'). Petrarch, Erasmus, Fuller and Dickinson added.</t>
+          <t>28 Oct 2026: Machiavelli, Bacon, La Bruyère, Vauvenargues and Chamfort added.</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G90"/>
+  <dimension ref="A1:G96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2301,7 +2308,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Enlightenment thinkers disagree. For Mill, happiness means pleasure and the absence of pain, and it is the measure of right and wrong, with everyone counting equally. For Kant, happiness is too vague to guide us: morality is about becoming worthy of it. For du Châtelet, it depends on health, passions and freedom from prejudice.</t>
+          <t>Enlightenment thinkers disagree. For Mill, happiness means pleasure and the absence of pain, and it is the measure of right and wrong, with everyone counting equally. For Kant, happiness is too vague to guide us: morality is about becoming worthy of it. For du Châtelet, it depends on health, passions and freedom from prejudice. For Rousseau, lasting happiness is not made for a world that always changes, so we should enjoy contentment when it comes.</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -2319,7 +2326,11 @@
           <t>Updated</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr"/>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>28 Oct 2026: Rousseau added (new thought).</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -2367,7 +2378,7 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>In On Liberty, Mill argues that people should be free to think, speak and live as they choose, as long as they do not harm others. Freedom lets each person find their own way, and lets new ideas start anywhere.</t>
+          <t>Enlightenment thinkers saw freedom in different ways. For Locke, good laws protect it from other people's arbitrary will; for Rousseau, it means never being made to do what we do not want, and people are born free yet everywhere in chains; for Mill, in On Liberty, people should be free to think, speak and live as they choose, as long as they do not harm others.</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -2385,7 +2396,11 @@
           <t>Updated</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr"/>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>28 Oct 2026: Locke and Rousseau added (new thoughts).</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -2466,7 +2481,7 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Strong feelings and desires. Spinoza called being ruled by them 'bondage' and believed understanding them sets us free; Hume, by contrast, thought reason can only serve the passions, never rule them.</t>
+          <t>Strong feelings and desires. Spinoza called being ruled by them 'bondage' and believed understanding them sets us free; Hume thought reason can only serve the passions, never rule them; Diderot defended them: only great passions, he wrote, raise us to great things.</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
@@ -2481,10 +2496,14 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="inlineStr"/>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>28 Oct 2026: Diderot added (new thought).</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -2862,7 +2881,7 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>From the French essai, 'attempt' or 'trial'. Montaigne used the word for his short pieces in which he tests his judgment on any subject, starting with himself. He made it a new literary form.</t>
+          <t>From the French essai, 'attempt' or 'trial'. Montaigne used the word for his short pieces in which he tests his judgment on any subject, starting with himself, and made it a new literary form. Francis Bacon took up the word for his own Essays, first published in 1597.</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
@@ -2877,10 +2896,14 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="G51" s="5" t="inlineStr"/>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>28 Oct 2026: Bacon added (new thoughts).</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -2895,7 +2918,7 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>A short, sharp saying that sums up a truth about human behaviour. La Rochefoucauld's maxims are famous for exposing vanity and self-love (amour-propre) behind our good actions.</t>
+          <t>A short, sharp saying that sums up a truth about human behaviour. La Rochefoucauld's maxims are famous for exposing vanity and self-love (amour-propre) behind our good actions. In the 18th century Vauvenargues gave the form a warmer voice, trusting feeling, while Chamfort sharpened it into social satire.</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
@@ -2910,10 +2933,14 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="G52" s="5" t="inlineStr"/>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>28 Oct 2026: Vauvenargues and Chamfort added (new thoughts).</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
@@ -4168,6 +4195,228 @@
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>Enlightenment Ethics</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Tolerance</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>Accepting that others may believe and live differently. It was Voltaire's great cause: after Europe's long wars over doctrine, he argued that since we are all weak and mistaken, we should forgive one another's errors. Mill extended it to unusual characters and ways of life.</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>tolerance</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Toleration</t>
+        </is>
+      </c>
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>Enlightenment Ethics</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Prejudice</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>An opinion held without judgement, usually picked up in childhood before we could weigh it. Voltaire adds that some prejudices are good: the ones our judgement confirms once we reason. Du Châtelet counted freedom from prejudice as a source of happiness.</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>prejudice, prejudices</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Prejudice</t>
+        </is>
+      </c>
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>Enlightenment Ethics</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Social contract</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>The idea that a state rests on an agreement among the people it governs. Hobbes, Locke and Rousseau gave it different forms: for Hobbes, people give up some freedom for safety; for Locke, government must protect life, liberty and property; for Rousseau, citizens together make the laws they obey.</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>Social Contract, social contract</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Social_contract</t>
+        </is>
+      </c>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
+        <is>
+          <t>Enlightenment Ethics</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>Commonwealth</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Hobbes's word for an organised state, made when people agree to live under a common power. In Leviathan he argues that only such a power brings peace, and with peace the leisure to think.</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>Common-wealth, Common-wealths, commonwealth</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Commonwealth</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t>Enlightenment Ethics</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Citizen of the world</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>Someone loyal to humanity as a whole rather than to one country. Voltaire ends his article on the homeland with this ideal; the phrase goes back to the ancient Greek thinker Diogenes.</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>citizen of the universe, citizen of the world</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Cosmopolitanism</t>
+        </is>
+      </c>
+      <c r="F95" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>Enlightenment Ethics</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>Diderot effect</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>The modern name, given long after Diderot, for a chain of new wants: one new possession makes everything around it look shabby, so we replace that too. It comes from his essay on his new dressing gown.</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>Diderot effect</t>
+        </is>
+      </c>
+      <c r="E96" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Diderot_effect</t>
+        </is>
+      </c>
+      <c r="F96" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G90"/>
@@ -4181,7 +4430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F161"/>
+  <dimension ref="A1:F182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6197,7 +6446,7 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>A Treatise of Human Nature, Treatise</t>
+          <t>A Treatise of Human Nature, Treatise of Human Nature</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
@@ -6207,10 +6456,14 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="F72" s="5" t="inlineStr"/>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>28 Oct 2026: no longer opens on the bare word 'Treatise' (it showed on Locke's Second Treatise).</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
@@ -8703,6 +8956,678 @@
         </is>
       </c>
       <c r="F161" s="5" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="5" t="inlineStr">
+        <is>
+          <t>Niccolò Machiavelli</t>
+        </is>
+      </c>
+      <c r="B162" s="5" t="inlineStr">
+        <is>
+          <t>A Florentine diplomat and writer (1469–1527). After the Medici returned to power in 1512 and removed him from office, he wrote The Prince, a blunt guide to how rulers win and keep power, published in 1532, after his death.</t>
+        </is>
+      </c>
+      <c r="C162" s="5" t="inlineStr">
+        <is>
+          <t>Niccolò Machiavelli, Machiavelli</t>
+        </is>
+      </c>
+      <c r="D162" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Niccolò_Machiavelli</t>
+        </is>
+      </c>
+      <c r="E162" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F162" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="inlineStr">
+        <is>
+          <t>Francis Bacon</t>
+        </is>
+      </c>
+      <c r="B163" s="5" t="inlineStr">
+        <is>
+          <t>An English statesman and philosopher (1561–1626), born in London, who rose to Lord Chancellor before his fall in 1621. Often called the father of empiricism, he urged that knowledge be built on careful observation. His Essays grew from 10 in 1597 to 58 in 1625.</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>Francis Bacon, Bacon</t>
+        </is>
+      </c>
+      <c r="D163" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Francis_Bacon</t>
+        </is>
+      </c>
+      <c r="E163" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F163" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="5" t="inlineStr">
+        <is>
+          <t>Voltaire</t>
+        </is>
+      </c>
+      <c r="B164" s="5" t="inlineStr">
+        <is>
+          <t>The pen name of François-Marie Arouet (1694–1778), the best-known writer of the French Enlightenment, born and died in Paris. He campaigned for tolerance and freedom of thought, and spent most of his last twenty years at Ferney, near Geneva.</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>Voltaire</t>
+        </is>
+      </c>
+      <c r="D164" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Voltaire</t>
+        </is>
+      </c>
+      <c r="E164" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F164" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="5" t="inlineStr">
+        <is>
+          <t>Jean-Jacques Rousseau</t>
+        </is>
+      </c>
+      <c r="B165" s="5" t="inlineStr">
+        <is>
+          <t>A writer and philosopher (1712–1778), born in Geneva, who lived mostly in France. When The Social Contract and Emile came out in 1762, both were banned and burned, and he fled to Switzerland. His ideas later inspired the French Revolution.</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>Jean-Jacques Rousseau, Rousseau</t>
+        </is>
+      </c>
+      <c r="D165" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Jean-Jacques_Rousseau</t>
+        </is>
+      </c>
+      <c r="E165" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F165" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="5" t="inlineStr">
+        <is>
+          <t>Thomas Hobbes</t>
+        </is>
+      </c>
+      <c r="B166" s="5" t="inlineStr">
+        <is>
+          <t>An English philosopher (1588–1679), born in Malmesbury. He wrote Leviathan (1651) in exile in Paris, arguing that without a common power life would be 'solitary, poor, nasty, brutish, and short'.</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>Thomas Hobbes, Hobbes</t>
+        </is>
+      </c>
+      <c r="D166" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Thomas_Hobbes</t>
+        </is>
+      </c>
+      <c r="E166" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F166" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="5" t="inlineStr">
+        <is>
+          <t>John Locke</t>
+        </is>
+      </c>
+      <c r="B167" s="5" t="inlineStr">
+        <is>
+          <t>An English philosopher (1632–1704). He argued that the mind starts as a blank slate filled by experience, and that governments exist to protect people's natural rights to life, liberty and property.</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>John Locke, Locke</t>
+        </is>
+      </c>
+      <c r="D167" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/John_Locke</t>
+        </is>
+      </c>
+      <c r="E167" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F167" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="5" t="inlineStr">
+        <is>
+          <t>Jean de La Bruyère</t>
+        </is>
+      </c>
+      <c r="B168" s="5" t="inlineStr">
+        <is>
+          <t>A French writer (1645–1696), born in Paris, who was a tutor in the household of the Prince de Condé. His Characters, first published in 1688, are sharp portraits and remarks on the people of his time.</t>
+        </is>
+      </c>
+      <c r="C168" s="5" t="inlineStr">
+        <is>
+          <t>Jean de La Bruyère, La Bruyère</t>
+        </is>
+      </c>
+      <c r="D168" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Jean_de_La_Bruyère</t>
+        </is>
+      </c>
+      <c r="E168" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F168" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="5" t="inlineStr">
+        <is>
+          <t>Nicolas Chamfort</t>
+        </is>
+      </c>
+      <c r="B169" s="5" t="inlineStr">
+        <is>
+          <t>A French playwright and wit (1741–1794), elected to the Académie française in 1781. He welcomed the Revolution, was later imprisoned for criticising its excesses, and died in Paris in 1794. His maxims were published after his death.</t>
+        </is>
+      </c>
+      <c r="C169" s="5" t="inlineStr">
+        <is>
+          <t>Nicolas Chamfort, Chamfort</t>
+        </is>
+      </c>
+      <c r="D169" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Nicolas_Chamfort</t>
+        </is>
+      </c>
+      <c r="E169" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F169" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="5" t="inlineStr">
+        <is>
+          <t>Vauvenargues</t>
+        </is>
+      </c>
+      <c r="B170" s="5" t="inlineStr">
+        <is>
+          <t>Luc de Clapiers, marquis de Vauvenargues (1715–1747), a French soldier and moralist born in Aix-en-Provence. Broken in health by the retreat from Prague in 1742, he turned to writing; his Reflections and Maxims appeared in 1746, a year before his death. Voltaire was a close friend.</t>
+        </is>
+      </c>
+      <c r="C170" s="5" t="inlineStr">
+        <is>
+          <t>Vauvenargues</t>
+        </is>
+      </c>
+      <c r="D170" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Luc_de_Clapiers,_marquis_de_Vauvenargues</t>
+        </is>
+      </c>
+      <c r="E170" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F170" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="5" t="inlineStr">
+        <is>
+          <t>Denis Diderot</t>
+        </is>
+      </c>
+      <c r="B171" s="5" t="inlineStr">
+        <is>
+          <t>A French writer and philosopher (1713–1784), born in Langres, and chief editor of the Encyclopédie, the great Enlightenment survey of knowledge. He was jailed at Vincennes in 1749 for his writings.</t>
+        </is>
+      </c>
+      <c r="C171" s="5" t="inlineStr">
+        <is>
+          <t>Denis Diderot, Diderot</t>
+        </is>
+      </c>
+      <c r="D171" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Denis_Diderot</t>
+        </is>
+      </c>
+      <c r="E171" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F171" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="5" t="inlineStr">
+        <is>
+          <t>Candide</t>
+        </is>
+      </c>
+      <c r="B172" s="5" t="inlineStr">
+        <is>
+          <t>Voltaire's comic novel of 1759. Its young hero is taught that all is for the best, then lives through war, shipwreck and earthquake, and ends by tending his garden.</t>
+        </is>
+      </c>
+      <c r="C172" s="5" t="inlineStr">
+        <is>
+          <t>Candide</t>
+        </is>
+      </c>
+      <c r="D172" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Candide</t>
+        </is>
+      </c>
+      <c r="E172" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F172" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="5" t="inlineStr">
+        <is>
+          <t>Zadig</t>
+        </is>
+      </c>
+      <c r="B173" s="5" t="inlineStr">
+        <is>
+          <t>A philosophical tale by Voltaire (1748) about a wise young man in ancient Babylon whose fortunes rise and fall.</t>
+        </is>
+      </c>
+      <c r="C173" s="5" t="inlineStr">
+        <is>
+          <t>Zadig</t>
+        </is>
+      </c>
+      <c r="D173" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Zadig</t>
+        </is>
+      </c>
+      <c r="E173" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F173" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="5" t="inlineStr">
+        <is>
+          <t>Philosophical Dictionary</t>
+        </is>
+      </c>
+      <c r="B174" s="5" t="inlineStr">
+        <is>
+          <t>Voltaire's pocket dictionary of short, sharp articles (1764), on subjects from friendship to tolerance.</t>
+        </is>
+      </c>
+      <c r="C174" s="5" t="inlineStr">
+        <is>
+          <t>Philosophical Dictionary</t>
+        </is>
+      </c>
+      <c r="D174" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Dictionnaire_philosophique</t>
+        </is>
+      </c>
+      <c r="E174" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F174" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="5" t="inlineStr">
+        <is>
+          <t>Emile</t>
+        </is>
+      </c>
+      <c r="B175" s="5" t="inlineStr">
+        <is>
+          <t>Rousseau's long book on education (1762), which follows an imaginary boy from birth to adulthood. It was banned and burned soon after it appeared.</t>
+        </is>
+      </c>
+      <c r="C175" s="5" t="inlineStr">
+        <is>
+          <t>Emile</t>
+        </is>
+      </c>
+      <c r="D175" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Emile,_or_On_Education</t>
+        </is>
+      </c>
+      <c r="E175" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F175" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="5" t="inlineStr">
+        <is>
+          <t>Discourse on Inequality</t>
+        </is>
+      </c>
+      <c r="B176" s="5" t="inlineStr">
+        <is>
+          <t>Rousseau's essay of 1755 on how inequality began, starting with the first person who fenced off a piece of land and said 'This is mine'.</t>
+        </is>
+      </c>
+      <c r="C176" s="5" t="inlineStr">
+        <is>
+          <t>Discourse on Inequality</t>
+        </is>
+      </c>
+      <c r="D176" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Discourse_on_Inequality</t>
+        </is>
+      </c>
+      <c r="E176" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F176" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="5" t="inlineStr">
+        <is>
+          <t>Reveries of the Solitary Walker</t>
+        </is>
+      </c>
+      <c r="B177" s="5" t="inlineStr">
+        <is>
+          <t>Rousseau's last work: ten 'walks' of reflection, written from 1776 and left unfinished at his death in 1778.</t>
+        </is>
+      </c>
+      <c r="C177" s="5" t="inlineStr">
+        <is>
+          <t>Reveries of the Solitary Walker, Reveries</t>
+        </is>
+      </c>
+      <c r="D177" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Reveries_of_the_Solitary_Walker</t>
+        </is>
+      </c>
+      <c r="E177" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F177" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="5" t="inlineStr">
+        <is>
+          <t>Leviathan</t>
+        </is>
+      </c>
+      <c r="B178" s="5" t="inlineStr">
+        <is>
+          <t>Hobbes's book of 1651, named after a giant sea monster, on why people need a strong common power to live in peace.</t>
+        </is>
+      </c>
+      <c r="C178" s="5" t="inlineStr">
+        <is>
+          <t>Leviathan</t>
+        </is>
+      </c>
+      <c r="D178" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Leviathan_(Hobbes_book)</t>
+        </is>
+      </c>
+      <c r="E178" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F178" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="5" t="inlineStr">
+        <is>
+          <t>An Essay Concerning Human Understanding</t>
+        </is>
+      </c>
+      <c r="B179" s="5" t="inlineStr">
+        <is>
+          <t>Locke's great book on knowledge (dated 1690), arguing that all our ideas come from experience.</t>
+        </is>
+      </c>
+      <c r="C179" s="5" t="inlineStr">
+        <is>
+          <t>An Essay Concerning Human Understanding, Essay Concerning Human Understanding</t>
+        </is>
+      </c>
+      <c r="D179" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/An_Essay_Concerning_Human_Understanding</t>
+        </is>
+      </c>
+      <c r="E179" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F179" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="5" t="inlineStr">
+        <is>
+          <t>Second Treatise of Government</t>
+        </is>
+      </c>
+      <c r="B180" s="5" t="inlineStr">
+        <is>
+          <t>The second of Locke's Two Treatises of Government (dated 1690), on why governments exist: to protect the lives, liberty and property of the people.</t>
+        </is>
+      </c>
+      <c r="C180" s="5" t="inlineStr">
+        <is>
+          <t>Second Treatise of Government, Second Treatise</t>
+        </is>
+      </c>
+      <c r="D180" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Two_Treatises_of_Government</t>
+        </is>
+      </c>
+      <c r="E180" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F180" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="5" t="inlineStr">
+        <is>
+          <t>Philosophical Thoughts</t>
+        </is>
+      </c>
+      <c r="B181" s="5" t="inlineStr">
+        <is>
+          <t>Diderot's first original book (1746): short numbered thoughts that open with a defence of the passions.</t>
+        </is>
+      </c>
+      <c r="C181" s="5" t="inlineStr">
+        <is>
+          <t>Philosophical Thoughts</t>
+        </is>
+      </c>
+      <c r="D181" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Philosophical_Thoughts</t>
+        </is>
+      </c>
+      <c r="E181" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F181" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="5" t="inlineStr">
+        <is>
+          <t>Regrets on My Old Dressing Gown</t>
+        </is>
+      </c>
+      <c r="B182" s="5" t="inlineStr">
+        <is>
+          <t>A playful essay by Diderot (1772) about how one new possession, a scarlet dressing gown, led him to replace everything around it.</t>
+        </is>
+      </c>
+      <c r="C182" s="5" t="inlineStr">
+        <is>
+          <t>Regrets on My Old Dressing Gown</t>
+        </is>
+      </c>
+      <c r="D182" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Diderot_effect</t>
+        </is>
+      </c>
+      <c r="E182" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F182" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F161"/>
@@ -8716,7 +9641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -8834,9 +9759,9 @@
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Blaise Pascal and Simone Weil · Existential Thought
-Émilie du Châtelet · Enlightenment Ethics
-François de La Rochefoucauld · Humanists and Essayists
-Pascal's notes were published after his death as the Pensées. Du Châtelet was born here in 1706, and La Rochefoucauld's Maxims came out here in 1665. Simone Weil was born here in 1909.</t>
+Émilie du Châtelet, Voltaire and Denis Diderot · Enlightenment Ethics
+François de La Rochefoucauld, Jean de La Bruyère and Nicolas Chamfort · Humanists and Essayists
+Pascal's notes were published after his death as the Pensées. Du Châtelet was born here in 1706 and Voltaire in 1694; Diderot edited the Encyclopédie here. La Rochefoucauld's Maxims came out here in 1665, La Bruyère was born here in 1645, and Chamfort died here in 1794. Simone Weil was born here in 1909.</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -8849,7 +9774,11 @@
           <t>Updated</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>28 Oct 2026: Voltaire, Diderot, La Bruyère and Chamfort added.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -8893,8 +9822,8 @@
       <c r="C6" s="3" t="inlineStr">
         <is>
           <t>John Stuart Mill and Mary Wollstonecraft · Enlightenment Ethics
-George Eliot · Humanists and Essayists
-Mill was born here in 1806. Wollstonecraft lived and wrote here, and published A Vindication of the Rights of Woman in 1792. George Eliot also lived and wrote in London.</t>
+George Eliot and Francis Bacon · Humanists and Essayists
+Mill was born here in 1806. Wollstonecraft lived and wrote here, and published A Vindication of the Rights of Woman in 1792. George Eliot also lived and wrote in London. Francis Bacon was born here in 1561.</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -8907,7 +9836,11 @@
           <t>Updated</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>28 Oct 2026: Bacon added.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -9546,6 +10479,138 @@
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Europe &amp; the Mediterranean</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Florence</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Niccolò Machiavelli · Humanists and Essayists
+Machiavelli was born here in 1469 and served the Florentine Republic from 1498 to 1512. Removed from office when the Medici returned, he wrote The Prince on his farm near San Casciano, outside the city.</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Niccolò_Machiavelli</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia. The map needs a dot here (tools/make_maps.py).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Europe &amp; the Mediterranean</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Geneva</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Jean-Jacques Rousseau and Voltaire · Enlightenment Ethics
+Rousseau was born here in 1712. Voltaire spent most of his last twenty years at Ferney, just outside the city.</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Geneva</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia. The map needs a dot here (tools/make_maps.py).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Europe &amp; the Mediterranean</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Malmesbury and Wrington</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Thomas Hobbes and John Locke · Enlightenment Ethics
+Hobbes was born in Malmesbury, Wiltshire, in 1588, and Locke in Wrington, Somerset, in 1632. Hobbes wrote Leviathan in exile in Paris; Locke spent years in exile in the Dutch Republic from 1683.</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Thomas_Hobbes</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia. The map needs a dot here (tools/make_maps.py).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Europe &amp; the Mediterranean</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Aix-en-Provence</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Vauvenargues · Humanists and Essayists
+Vauvenargues was born here in 1715. After years as a soldier he settled in Paris, where he died in 1747.</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Luc_de_Clapiers,_marquis_de_Vauvenargues</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Added 28 Oct 2026 for the 31 new thoughts; checked against Wikipedia. The map needs a dot here (tools/make_maps.py).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F28"/>

</xml_diff>